<commit_message>
Adding new models and model outputs
</commit_message>
<xml_diff>
--- a/data_raw/Thrown together GEF-8 numbers.xlsx
+++ b/data_raw/Thrown together GEF-8 numbers.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://worldbankgroup-my.sharepoint.com/personal/swyatt_thegef_org/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/samaramanzin/Desktop/cali_fund/data_raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5C1B4FE9-B91E-4408-853E-14B2CC412014}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90D06DDD-C69B-5E42-9D0E-09D966A6B855}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2E359720-BDD9-49A0-BB6D-879A737A4040}"/>
+    <workbookView xWindow="4280" yWindow="600" windowWidth="24520" windowHeight="15720" xr2:uid="{2E359720-BDD9-49A0-BB6D-879A737A4040}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1622,7 +1622,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -1707,7 +1707,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -2044,17 +2044,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2065395D-AABA-4F95-9E35-A4E0775BAA98}">
   <dimension ref="A1:E276"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="26.42578125" customWidth="1"/>
-    <col min="2" max="2" width="42.85546875" customWidth="1"/>
-    <col min="3" max="3" width="17.7109375" customWidth="1"/>
-    <col min="4" max="4" width="25.5703125" customWidth="1"/>
-    <col min="5" max="5" width="21.28515625" customWidth="1"/>
+    <col min="1" max="1" width="26.5" customWidth="1"/>
+    <col min="2" max="2" width="42.83203125" customWidth="1"/>
+    <col min="3" max="3" width="17.6640625" customWidth="1"/>
+    <col min="4" max="4" width="25.5" customWidth="1"/>
+    <col min="5" max="5" width="21.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -2068,7 +2068,7 @@
         <v>525</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -2086,7 +2086,7 @@
         <v>0.21714266689251038</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -2104,7 +2104,7 @@
         <v>6.0233380608775575E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -2122,7 +2122,7 @@
         <v>0.20839759547231637</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -2140,7 +2140,7 @@
         <v>3.4257035077481512E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -2158,7 +2158,7 @@
         <v>1.1427718349100224E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -2176,7 +2176,7 @@
         <v>0.61071820601882565</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -2194,7 +2194,7 @@
         <v>2.5475959199010467E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -2212,7 +2212,7 @@
         <v>0.2309302620122364</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>18</v>
       </c>
@@ -2230,7 +2230,7 @@
         <v>4.3313568202959708E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>20</v>
       </c>
@@ -2248,7 +2248,7 @@
         <v>1.3220040700709368</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>22</v>
       </c>
@@ -2266,7 +2266,7 @@
         <v>3.6681895121167249E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>24</v>
       </c>
@@ -2284,7 +2284,7 @@
         <v>3.5988668032775922E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>26</v>
       </c>
@@ -2302,7 +2302,7 @@
         <v>4.9210278363647975</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>28</v>
       </c>
@@ -2320,7 +2320,7 @@
         <v>5.1150495916130252E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>30</v>
       </c>
@@ -2338,7 +2338,7 @@
         <v>4.9571713904422179E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>32</v>
       </c>
@@ -2356,7 +2356,7 @@
         <v>0.27567952292026399</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>34</v>
       </c>
@@ -2374,7 +2374,7 @@
         <v>1.5120131174547406E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>36</v>
       </c>
@@ -2392,7 +2392,7 @@
         <v>0.14084999444145968</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>38</v>
       </c>
@@ -2410,7 +2410,7 @@
         <v>4.7838843577585909E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>40</v>
       </c>
@@ -2428,7 +2428,7 @@
         <v>2.3715767696354008E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>42</v>
       </c>
@@ -2446,7 +2446,7 @@
         <v>2.4023160888868841E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>44</v>
       </c>
@@ -2464,7 +2464,7 @@
         <v>0.11754130767456389</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>46</v>
       </c>
@@ -2482,7 +2482,7 @@
         <v>5.7498841847122416E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>48</v>
       </c>
@@ -2500,7 +2500,7 @@
         <v>7.576198338838544E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>50</v>
       </c>
@@ -2518,7 +2518,7 @@
         <v>8.4562106307997459E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>52</v>
       </c>
@@ -2536,7 +2536,7 @@
         <v>1.017301421742737</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>54</v>
       </c>
@@ -2554,7 +2554,7 @@
         <v>4.190623612089308E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>56</v>
       </c>
@@ -2572,7 +2572,7 @@
         <v>3.7822834334671707E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>58</v>
       </c>
@@ -2590,7 +2590,7 @@
         <v>0.14554526936258327</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>60</v>
       </c>
@@ -2608,7 +2608,7 @@
         <v>2.1964180801455239E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>62</v>
       </c>
@@ -2626,7 +2626,7 @@
         <v>5.9266621901072973</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>64</v>
       </c>
@@ -2644,7 +2644,7 @@
         <v>5.8597504187962876E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>66</v>
       </c>
@@ -2662,7 +2662,7 @@
         <v>4.4628661030076781E-2</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>68</v>
       </c>
@@ -2680,7 +2680,7 @@
         <v>3.399842873737273E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>70</v>
       </c>
@@ -2698,7 +2698,7 @@
         <v>7.6244815609067901E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>72</v>
       </c>
@@ -2716,7 +2716,7 @@
         <v>4.7760849311338727E-2</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>74</v>
       </c>
@@ -2734,7 +2734,7 @@
         <v>5.4755557402506178E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>76</v>
       </c>
@@ -2752,7 +2752,7 @@
         <v>0.22327849415061088</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>78</v>
       </c>
@@ -2770,7 +2770,7 @@
         <v>0.90962190721941238</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>80</v>
       </c>
@@ -2788,7 +2788,7 @@
         <v>1.1714328644347676</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>82</v>
       </c>
@@ -2806,7 +2806,7 @@
         <v>0.32806053175448541</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>84</v>
       </c>
@@ -2824,7 +2824,7 @@
         <v>4.3377226294962518E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>86</v>
       </c>
@@ -2842,7 +2842,7 @@
         <v>0.13427215655910935</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>88</v>
       </c>
@@ -2860,7 +2860,7 @@
         <v>0.13040393787944471</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>90</v>
       </c>
@@ -2878,7 +2878,7 @@
         <v>0.89615865394973038</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>92</v>
       </c>
@@ -2896,7 +2896,7 @@
         <v>3.2339355098198306</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>94</v>
       </c>
@@ -2914,7 +2914,7 @@
         <v>7.2115783440141537E-2</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>96</v>
       </c>
@@ -2932,7 +2932,7 @@
         <v>5.6968197894353659E-2</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>98</v>
       </c>
@@ -2950,7 +2950,7 @@
         <v>3.1568954016350903E-2</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>100</v>
       </c>
@@ -2968,7 +2968,7 @@
         <v>3.569997758047712</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>102</v>
       </c>
@@ -2986,7 +2986,7 @@
         <v>0.11948312617212836</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>104</v>
       </c>
@@ -3004,7 +3004,7 @@
         <v>0.15714973708954372</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>106</v>
       </c>
@@ -3022,7 +3022,7 @@
         <v>8.8099987708388852E-2</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>108</v>
       </c>
@@ -3040,7 +3040,7 @@
         <v>0.72966936034028707</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>110</v>
       </c>
@@ -3058,7 +3058,7 @@
         <v>0.30748084140860432</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>112</v>
       </c>
@@ -3076,7 +3076,7 @@
         <v>6.8166890911777661E-2</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>114</v>
       </c>
@@ -3094,7 +3094,7 @@
         <v>0.7513299690879387</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>116</v>
       </c>
@@ -3112,7 +3112,7 @@
         <v>4.4143772849547014E-2</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>118</v>
       </c>
@@ -3130,7 +3130,7 @@
         <v>3.9300742825049306E-2</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>120</v>
       </c>
@@ -3148,7 +3148,7 @@
         <v>3.8063651920152618E-2</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>122</v>
       </c>
@@ -3166,7 +3166,7 @@
         <v>6.5583406767860369E-2</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>124</v>
       </c>
@@ -3184,7 +3184,7 @@
         <v>1.2080321734474946</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>126</v>
       </c>
@@ -3202,7 +3202,7 @@
         <v>4.0802527129792814E-2</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>128</v>
       </c>
@@ -3220,7 +3220,7 @@
         <v>5.2648531094903493E-2</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>130</v>
       </c>
@@ -3238,7 +3238,7 @@
         <v>6.9321189385039075E-2</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>132</v>
       </c>
@@ -3256,7 +3256,7 @@
         <v>0.36751870726116681</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>134</v>
       </c>
@@ -3274,7 +3274,7 @@
         <v>2.2015285591018459</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>136</v>
       </c>
@@ -3292,7 +3292,7 @@
         <v>0.23930590614354835</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>138</v>
       </c>
@@ -3310,7 +3310,7 @@
         <v>9.2254883131574233E-2</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>140</v>
       </c>
@@ -3328,7 +3328,7 @@
         <v>0.11258233360887945</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>142</v>
       </c>
@@ -3346,7 +3346,7 @@
         <v>0.13361237574847426</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>144</v>
       </c>
@@ -3364,7 +3364,7 @@
         <v>2.478503498205881E-2</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>146</v>
       </c>
@@ -3382,7 +3382,7 @@
         <v>0.6483546981490349</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>148</v>
       </c>
@@ -3400,7 +3400,7 @@
         <v>6.9002088311971035E-2</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>150</v>
       </c>
@@ -3418,7 +3418,7 @@
         <v>6.191952004570303E-2</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>152</v>
       </c>
@@ -3436,7 +3436,7 @@
         <v>0.31993311272635211</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>154</v>
       </c>
@@ -3454,7 +3454,7 @@
         <v>2.6059080685375588E-2</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>156</v>
       </c>
@@ -3472,7 +3472,7 @@
         <v>0.24752942425549429</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>158</v>
       </c>
@@ -3490,7 +3490,7 @@
         <v>9.6983307020745341E-2</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>160</v>
       </c>
@@ -3508,7 +3508,7 @@
         <v>0.47458710991966746</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>162</v>
       </c>
@@ -3526,7 +3526,7 @@
         <v>0.24604086223579646</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>164</v>
       </c>
@@ -3544,7 +3544,7 @@
         <v>3.8675289691325582E-2</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>166</v>
       </c>
@@ -3562,7 +3562,7 @@
         <v>6.4646727359481848E-2</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>168</v>
       </c>
@@ -3580,7 +3580,7 @@
         <v>7.8922104644424895E-2</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>170</v>
       </c>
@@ -3598,7 +3598,7 @@
         <v>0.22120217140697351</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>172</v>
       </c>
@@ -3616,7 +3616,7 @@
         <v>9.6087113738893039E-3</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>174</v>
       </c>
@@ -3634,7 +3634,7 @@
         <v>0.22853399776139505</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>176</v>
       </c>
@@ -3652,7 +3652,7 @@
         <v>0.11628035980328763</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>178</v>
       </c>
@@ -3670,7 +3670,7 @@
         <v>5.7910399114206271E-2</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>180</v>
       </c>
@@ -3688,7 +3688,7 @@
         <v>0.1045121289887733</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>182</v>
       </c>
@@ -3706,7 +3706,7 @@
         <v>5.4179601016288187E-2</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>184</v>
       </c>
@@ -3724,7 +3724,7 @@
         <v>0.65650851866190751</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>186</v>
       </c>
@@ -3742,7 +3742,7 @@
         <v>1.275415954222496E-2</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>188</v>
       </c>
@@ -3760,7 +3760,7 @@
         <v>0.20185193637547419</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>190</v>
       </c>
@@ -3778,7 +3778,7 @@
         <v>6.602453043609402E-2</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>192</v>
       </c>
@@ -3796,7 +3796,7 @@
         <v>0.21684066049984702</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>194</v>
       </c>
@@ -3814,7 +3814,7 @@
         <v>0.43549476571005308</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>196</v>
       </c>
@@ -3832,7 +3832,7 @@
         <v>2.8792693833200621E-2</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>198</v>
       </c>
@@ -3850,7 +3850,7 @@
         <v>4.8226878515945099E-5</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>200</v>
       </c>
@@ -3868,7 +3868,7 @@
         <v>0.65040168177011526</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>202</v>
       </c>
@@ -3886,7 +3886,7 @@
         <v>1.7644192166440666E-2</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>204</v>
       </c>
@@ -3904,7 +3904,7 @@
         <v>1.7093182347622197E-2</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>206</v>
       </c>
@@ -3922,7 +3922,7 @@
         <v>0.10915772162363267</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>208</v>
       </c>
@@ -3940,7 +3940,7 @@
         <v>2.8501573774084537</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>210</v>
       </c>
@@ -3958,7 +3958,7 @@
         <v>6.5899578955005493</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>212</v>
       </c>
@@ -3976,7 +3976,7 @@
         <v>0.39990909569973632</v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>214</v>
       </c>
@@ -3994,7 +3994,7 @@
         <v>0.10816850673958699</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>216</v>
       </c>
@@ -4012,7 +4012,7 @@
         <v>7.6987210229233244E-2</v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>218</v>
       </c>
@@ -4030,7 +4030,7 @@
         <v>7.3150467894211573E-3</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>220</v>
       </c>
@@ -4048,7 +4048,7 @@
         <v>6.4447003864169156E-2</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
         <v>222</v>
       </c>
@@ -4066,7 +4066,7 @@
         <v>0.37750851528122598</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
         <v>224</v>
       </c>
@@ -4084,7 +4084,7 @@
         <v>0.28964585646645102</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
         <v>226</v>
       </c>
@@ -4102,7 +4102,7 @@
         <v>1.3369981684954326</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
         <v>228</v>
       </c>
@@ -4120,7 +4120,7 @@
         <v>1.3152219434207781E-2</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
         <v>230</v>
       </c>
@@ -4138,7 +4138,7 @@
         <v>3.8748077118185668E-2</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
         <v>232</v>
       </c>
@@ -4156,7 +4156,7 @@
         <v>0.32051584915821685</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
         <v>234</v>
       </c>
@@ -4174,7 +4174,7 @@
         <v>0.65570500393689124</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
         <v>236</v>
       </c>
@@ -4192,7 +4192,7 @@
         <v>0.14674361326655949</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
         <v>238</v>
       </c>
@@ -4210,7 +4210,7 @@
         <v>2.1037096937047001E-2</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
         <v>240</v>
       </c>
@@ -4228,7 +4228,7 @@
         <v>7.7730055573744516E-2</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
         <v>242</v>
       </c>
@@ -4246,7 +4246,7 @@
         <v>0.32364323637696857</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
         <v>244</v>
       </c>
@@ -4264,7 +4264,7 @@
         <v>1.4537727345722673E-2</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
         <v>246</v>
       </c>
@@ -4282,7 +4282,7 @@
         <v>3.3662381316235807E-2</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
         <v>248</v>
       </c>
@@ -4300,7 +4300,7 @@
         <v>3.037942261483717E-2</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
         <v>250</v>
       </c>
@@ -4318,7 +4318,7 @@
         <v>0.16709874172949579</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
         <v>252</v>
       </c>
@@ -4336,7 +4336,7 @@
         <v>0.13367922380688785</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
         <v>254</v>
       </c>
@@ -4354,7 +4354,7 @@
         <v>8.7488571862611494E-3</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
         <v>256</v>
       </c>
@@ -4372,7 +4372,7 @@
         <v>1.9693255867424354E-2</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
         <v>258</v>
       </c>
@@ -4390,7 +4390,7 @@
         <v>8.7294949826058794E-3</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
         <v>260</v>
       </c>
@@ -4408,7 +4408,7 @@
         <v>8.0981189560948592E-5</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
         <v>262</v>
       </c>
@@ -4426,7 +4426,7 @@
         <v>2.9005661536161997</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
         <v>264</v>
       </c>
@@ -4444,7 +4444,7 @@
         <v>0.16067202967043703</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
         <v>266</v>
       </c>
@@ -4462,7 +4462,7 @@
         <v>1.1042247494391777</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
         <v>268</v>
       </c>
@@ -4480,7 +4480,7 @@
         <v>9.9712550237900197E-2</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
         <v>270</v>
       </c>
@@ -4498,7 +4498,7 @@
         <v>0.11664070347268581</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
         <v>272</v>
       </c>
@@ -4516,7 +4516,7 @@
         <v>2.1157184815055949E-2</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
         <v>274</v>
       </c>
@@ -4534,7 +4534,7 @@
         <v>0.14266486338204773</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
         <v>276</v>
       </c>
@@ -4552,7 +4552,7 @@
         <v>8.5270998335120265E-2</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
         <v>278</v>
       </c>
@@ -4570,7 +4570,7 @@
         <v>9.9309400605036846E-2</v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
         <v>280</v>
       </c>
@@ -4588,7 +4588,7 @@
         <v>0.19326782634910536</v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A143" t="s">
         <v>282</v>
       </c>
@@ -4606,7 +4606,7 @@
         <v>3.8091049112778511E-2</v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A144" t="s">
         <v>284</v>
       </c>
@@ -4624,7 +4624,7 @@
         <v>4.484056807922701</v>
       </c>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A145" t="s">
         <v>286</v>
       </c>
@@ -4642,7 +4642,7 @@
         <v>0.25193684559227036</v>
       </c>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A146" t="s">
         <v>288</v>
       </c>
@@ -4660,7 +4660,7 @@
         <v>5.2997452234203818E-3</v>
       </c>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A147" t="s">
         <v>290</v>
       </c>
@@ -4678,7 +4678,7 @@
         <v>0.24452811010596204</v>
       </c>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A148" t="s">
         <v>292</v>
       </c>
@@ -4696,7 +4696,7 @@
         <v>3.6484295008701054E-2</v>
       </c>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A149" t="s">
         <v>294</v>
       </c>
@@ -4714,7 +4714,7 @@
         <v>1.6684739484619938E-2</v>
       </c>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A150" t="s">
         <v>296</v>
       </c>
@@ -4732,7 +4732,7 @@
         <v>0.21061114631789607</v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A151" t="s">
         <v>298</v>
       </c>
@@ -4750,7 +4750,7 @@
         <v>0.56606177290011206</v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A152" t="s">
         <v>300</v>
       </c>
@@ -4768,7 +4768,7 @@
         <v>0.80583180907337226</v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A153" t="s">
         <v>302</v>
       </c>
@@ -4786,7 +4786,7 @@
         <v>0.38954859768970435</v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A154" t="s">
         <v>304</v>
       </c>
@@ -4804,7 +4804,7 @@
         <v>2.3230260557015065E-2</v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A155" t="s">
         <v>306</v>
       </c>
@@ -4822,7 +4822,7 @@
         <v>0.23743763051135519</v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A156" t="s">
         <v>308</v>
       </c>
@@ -4840,7 +4840,7 @@
         <v>2.0516118538555631E-2</v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A157" t="s">
         <v>310</v>
       </c>
@@ -4858,7 +4858,7 @@
         <v>0.4038556819852912</v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A158" t="s">
         <v>312</v>
       </c>
@@ -4876,7 +4876,7 @@
         <v>1.0478422686125639</v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A159" t="s">
         <v>314</v>
       </c>
@@ -4894,7 +4894,7 @@
         <v>0.32474312954169116</v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A160" t="s">
         <v>316</v>
       </c>
@@ -4912,7 +4912,7 @@
         <v>7.5739205809050775E-2</v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A161" t="s">
         <v>318</v>
       </c>
@@ -4930,7 +4930,7 @@
         <v>0.45899978213569892</v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A162" t="s">
         <v>320</v>
       </c>
@@ -4948,7 +4948,7 @@
         <v>2.3200745740667009E-2</v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A163" t="s">
         <v>322</v>
       </c>
@@ -4966,7 +4966,7 @@
         <v>7.6155948848663835E-2</v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A164" t="s">
         <v>324</v>
       </c>
@@ -4984,7 +4984,7 @@
         <v>0.2516867743150123</v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A165" t="s">
         <v>326</v>
       </c>
@@ -5002,7 +5002,7 @@
         <v>0.2607188095213423</v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A166" t="s">
         <v>328</v>
       </c>
@@ -5020,7 +5020,7 @@
         <v>0.30314993528568629</v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A167" t="s">
         <v>330</v>
       </c>
@@ -5038,7 +5038,7 @@
         <v>0.12491669732433963</v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A168" t="s">
         <v>332</v>
       </c>
@@ -5056,7 +5056,7 @@
         <v>0.82623978437071854</v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A169" t="s">
         <v>334</v>
       </c>
@@ -5074,7 +5074,7 @@
         <v>2.2843182429685163</v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A170" t="s">
         <v>336</v>
       </c>
@@ -5092,7 +5092,7 @@
         <v>0.17082531596389833</v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A171" t="s">
         <v>338</v>
       </c>
@@ -5110,7 +5110,7 @@
         <v>2.7638844609611093</v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A172" t="s">
         <v>340</v>
       </c>
@@ -5128,7 +5128,7 @@
         <v>2.2264104728817156</v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A173" t="s">
         <v>342</v>
       </c>
@@ -5146,7 +5146,7 @@
         <v>3.9643534091198383E-2</v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A174" t="s">
         <v>344</v>
       </c>
@@ -5164,7 +5164,7 @@
         <v>6.2938880403692998E-2</v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A175" t="s">
         <v>346</v>
       </c>
@@ -5182,7 +5182,7 @@
         <v>0.23203665095714363</v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A176" t="s">
         <v>348</v>
       </c>
@@ -5200,7 +5200,7 @@
         <v>0.27329525803158183</v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A177" t="s">
         <v>350</v>
       </c>
@@ -5218,7 +5218,7 @@
         <v>2.0162155356625158E-2</v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A178" t="s">
         <v>352</v>
       </c>
@@ -5236,7 +5236,7 @@
         <v>0.1914596175794383</v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A179" t="s">
         <v>354</v>
       </c>
@@ -5254,7 +5254,7 @@
         <v>0.19529931603356324</v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A180" t="s">
         <v>356</v>
       </c>
@@ -5272,7 +5272,7 @@
         <v>2.7535746326912123E-3</v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A181" t="s">
         <v>358</v>
       </c>
@@ -5290,7 +5290,7 @@
         <v>0.10832708067522298</v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A182" t="s">
         <v>360</v>
       </c>
@@ -5308,7 +5308,7 @@
         <v>8.0723793646779493E-2</v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A183" t="s">
         <v>362</v>
       </c>
@@ -5326,7 +5326,7 @@
         <v>1.4161862420234566</v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A184" t="s">
         <v>364</v>
       </c>
@@ -5344,7 +5344,7 @@
         <v>7.913274533439732E-2</v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A185" t="s">
         <v>366</v>
       </c>
@@ -5362,7 +5362,7 @@
         <v>1.7640800695725711E-2</v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A186" t="s">
         <v>368</v>
       </c>
@@ -5380,7 +5380,7 @@
         <v>0.17829105451371746</v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A187" t="s">
         <v>370</v>
       </c>
@@ -5398,7 +5398,7 @@
         <v>1.8816520066093613E-2</v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A188" t="s">
         <v>372</v>
       </c>
@@ -5416,7 +5416,7 @@
         <v>7.8291766543169938E-2</v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A189" t="s">
         <v>374</v>
       </c>
@@ -5434,7 +5434,7 @@
         <v>1.0849420665189234E-2</v>
       </c>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A190" t="s">
         <v>376</v>
       </c>
@@ -5452,7 +5452,7 @@
         <v>1.3364031882417181E-2</v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A191" t="s">
         <v>378</v>
       </c>
@@ -5470,7 +5470,7 @@
         <v>6.4327175937778786E-2</v>
       </c>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A192" t="s">
         <v>380</v>
       </c>
@@ -5488,7 +5488,7 @@
         <v>7.8847138913454559E-2</v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A193" t="s">
         <v>382</v>
       </c>
@@ -5506,7 +5506,7 @@
         <v>1.1636953225770522E-2</v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A194" t="s">
         <v>384</v>
       </c>
@@ -5524,7 +5524,7 @@
         <v>0.16979738892359619</v>
       </c>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A195" t="s">
         <v>386</v>
       </c>
@@ -5542,7 +5542,7 @@
         <v>0.42976592791978152</v>
       </c>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A196" t="s">
         <v>388</v>
       </c>
@@ -5560,7 +5560,7 @@
         <v>0.2201428473973448</v>
       </c>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A197" t="s">
         <v>390</v>
       </c>
@@ -5578,7 +5578,7 @@
         <v>4.3830033869946057E-2</v>
       </c>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A198" t="s">
         <v>392</v>
       </c>
@@ -5596,7 +5596,7 @@
         <v>0.24118778860309781</v>
       </c>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A199" t="s">
         <v>394</v>
       </c>
@@ -5614,7 +5614,7 @@
         <v>0.11965602592265946</v>
       </c>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A200" t="s">
         <v>396</v>
       </c>
@@ -5632,7 +5632,7 @@
         <v>1.5693198601980318E-2</v>
       </c>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A201" t="s">
         <v>398</v>
       </c>
@@ -5650,7 +5650,7 @@
         <v>9.303772476929012E-3</v>
       </c>
     </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A202" t="s">
         <v>400</v>
       </c>
@@ -5668,7 +5668,7 @@
         <v>2.0219294393740216E-2</v>
       </c>
     </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A203" t="s">
         <v>402</v>
       </c>
@@ -5686,7 +5686,7 @@
         <v>3.4119019590617514E-2</v>
       </c>
     </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A204" t="s">
         <v>404</v>
       </c>
@@ -5704,7 +5704,7 @@
         <v>0.49584739876475881</v>
       </c>
     </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A205" t="s">
         <v>406</v>
       </c>
@@ -5722,7 +5722,7 @@
         <v>0.44657835166001741</v>
       </c>
     </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A206" t="s">
         <v>408</v>
       </c>
@@ -5740,7 +5740,7 @@
         <v>1.6393356057375237</v>
       </c>
     </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A207" t="s">
         <v>410</v>
       </c>
@@ -5758,7 +5758,7 @@
         <v>6.651398197328455E-2</v>
       </c>
     </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A208" t="s">
         <v>412</v>
       </c>
@@ -5776,7 +5776,7 @@
         <v>0.15645828198799391</v>
       </c>
     </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A209" t="s">
         <v>414</v>
       </c>
@@ -5794,7 +5794,7 @@
         <v>0.53145725994847104</v>
       </c>
     </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A210" t="s">
         <v>416</v>
       </c>
@@ -5812,7 +5812,7 @@
         <v>0.75433583880179234</v>
       </c>
     </row>
-    <row r="211" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A211" t="s">
         <v>418</v>
       </c>
@@ -5830,7 +5830,7 @@
         <v>3.6255506701430115E-2</v>
       </c>
     </row>
-    <row r="212" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A212" t="s">
         <v>420</v>
       </c>
@@ -5848,7 +5848,7 @@
         <v>0.21432074460415806</v>
       </c>
     </row>
-    <row r="213" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A213" t="s">
         <v>422</v>
       </c>
@@ -5866,7 +5866,7 @@
         <v>0.14613195889437391</v>
       </c>
     </row>
-    <row r="214" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A214" t="s">
         <v>424</v>
       </c>
@@ -5884,7 +5884,7 @@
         <v>2.8407877394567727E-2</v>
       </c>
     </row>
-    <row r="215" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A215" t="s">
         <v>426</v>
       </c>
@@ -5902,7 +5902,7 @@
         <v>2.8543734229583437E-2</v>
       </c>
     </row>
-    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A216" t="s">
         <v>428</v>
       </c>
@@ -5920,7 +5920,7 @@
         <v>7.224456397786834E-2</v>
       </c>
     </row>
-    <row r="217" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A217" t="s">
         <v>430</v>
       </c>
@@ -5938,7 +5938,7 @@
         <v>2.3243865557842795E-2</v>
       </c>
     </row>
-    <row r="218" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A218" t="s">
         <v>432</v>
       </c>
@@ -5956,7 +5956,7 @@
         <v>6.3982802061469057E-2</v>
       </c>
     </row>
-    <row r="219" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A219" t="s">
         <v>434</v>
       </c>
@@ -5974,7 +5974,7 @@
         <v>0.41898934547845501</v>
       </c>
     </row>
-    <row r="220" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A220" t="s">
         <v>436</v>
       </c>
@@ -5992,7 +5992,7 @@
         <v>5.9161323664261342E-2</v>
       </c>
     </row>
-    <row r="221" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A221" t="s">
         <v>438</v>
       </c>
@@ -6010,7 +6010,7 @@
         <v>0.18375254902205396</v>
       </c>
     </row>
-    <row r="222" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A222" t="s">
         <v>440</v>
       </c>
@@ -6028,7 +6028,7 @@
         <v>0.60054808497380319</v>
       </c>
     </row>
-    <row r="223" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A223" t="s">
         <v>442</v>
       </c>
@@ -6046,7 +6046,7 @@
         <v>2.9814466181134334E-2</v>
       </c>
     </row>
-    <row r="224" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A224" t="s">
         <v>444</v>
       </c>
@@ -6064,7 +6064,7 @@
         <v>8.6450375965008208E-2</v>
       </c>
     </row>
-    <row r="225" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A225" t="s">
         <v>446</v>
       </c>
@@ -6082,7 +6082,7 @@
         <v>5.4043884492273542E-2</v>
       </c>
     </row>
-    <row r="226" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A226" t="s">
         <v>448</v>
       </c>
@@ -6100,7 +6100,7 @@
         <v>2.7274016975327855E-2</v>
       </c>
     </row>
-    <row r="227" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A227" t="s">
         <v>450</v>
       </c>
@@ -6118,7 +6118,7 @@
         <v>0.15665854415534644</v>
       </c>
     </row>
-    <row r="228" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A228" t="s">
         <v>452</v>
       </c>
@@ -6136,7 +6136,7 @@
         <v>0.14336334819751628</v>
       </c>
     </row>
-    <row r="229" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A229" t="s">
         <v>454</v>
       </c>
@@ -6154,7 +6154,7 @@
         <v>0.10598653216375394</v>
       </c>
     </row>
-    <row r="230" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A230" t="s">
         <v>456</v>
       </c>
@@ -6172,7 +6172,7 @@
         <v>0.39356634188671741</v>
       </c>
     </row>
-    <row r="231" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A231" t="s">
         <v>458</v>
       </c>
@@ -6190,7 +6190,7 @@
         <v>9.9721674121135903E-2</v>
       </c>
     </row>
-    <row r="232" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A232" t="s">
         <v>460</v>
       </c>
@@ -6208,7 +6208,7 @@
         <v>3.5524894779127091E-2</v>
       </c>
     </row>
-    <row r="233" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A233" t="s">
         <v>462</v>
       </c>
@@ -6226,7 +6226,7 @@
         <v>3.9440387198290509E-2</v>
       </c>
     </row>
-    <row r="234" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A234" t="s">
         <v>464</v>
       </c>
@@ -6244,7 +6244,7 @@
         <v>0.21971318638114729</v>
       </c>
     </row>
-    <row r="235" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A235" t="s">
         <v>466</v>
       </c>
@@ -6262,7 +6262,7 @@
         <v>0.12270315665186847</v>
       </c>
     </row>
-    <row r="236" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A236" t="s">
         <v>468</v>
       </c>
@@ -6280,7 +6280,7 @@
         <v>6.9848564058067303E-2</v>
       </c>
     </row>
-    <row r="237" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A237" t="s">
         <v>470</v>
       </c>
@@ -6298,7 +6298,7 @@
         <v>0.16882924310721475</v>
       </c>
     </row>
-    <row r="238" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A238" t="s">
         <v>472</v>
       </c>
@@ -6316,7 +6316,7 @@
         <v>1.3600693247352373</v>
       </c>
     </row>
-    <row r="239" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A239" t="s">
         <v>474</v>
       </c>
@@ -6334,7 +6334,7 @@
         <v>7.7255215700405999E-2</v>
       </c>
     </row>
-    <row r="240" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A240" t="s">
         <v>476</v>
       </c>
@@ -6352,7 +6352,7 @@
         <v>4.2137622658441298</v>
       </c>
     </row>
-    <row r="241" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A241" t="s">
         <v>478</v>
       </c>
@@ -6370,7 +6370,7 @@
         <v>3.3628382005415305E-2</v>
       </c>
     </row>
-    <row r="242" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A242" t="s">
         <v>480</v>
       </c>
@@ -6388,7 +6388,7 @@
         <v>0.15368846641233541</v>
       </c>
     </row>
-    <row r="243" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A243" t="s">
         <v>482</v>
       </c>
@@ -6406,7 +6406,7 @@
         <v>8.27779677649607E-2</v>
       </c>
     </row>
-    <row r="244" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A244" t="s">
         <v>484</v>
       </c>
@@ -6424,7 +6424,7 @@
         <v>0.17219947294559074</v>
       </c>
     </row>
-    <row r="245" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A245" t="s">
         <v>486</v>
       </c>
@@ -6442,7 +6442,7 @@
         <v>1.8907129797128106</v>
       </c>
     </row>
-    <row r="246" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A246" t="s">
         <v>488</v>
       </c>
@@ -6460,7 +6460,7 @@
         <v>0.88360496126057408</v>
       </c>
     </row>
-    <row r="247" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A247" t="s">
         <v>490</v>
       </c>
@@ -6478,7 +6478,7 @@
         <v>2.7769361426721272E-2</v>
       </c>
     </row>
-    <row r="248" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A248" t="s">
         <v>492</v>
       </c>
@@ -6496,7 +6496,7 @@
         <v>6.7663113619187698E-2</v>
       </c>
     </row>
-    <row r="249" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A249" t="s">
         <v>494</v>
       </c>
@@ -6514,7 +6514,7 @@
         <v>0.35033783669063323</v>
       </c>
     </row>
-    <row r="250" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A250" t="s">
         <v>496</v>
       </c>
@@ -6532,7 +6532,7 @@
         <v>0.30527801715082492</v>
       </c>
     </row>
-    <row r="251" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A251" t="s">
         <v>498</v>
       </c>
@@ -6550,7 +6550,7 @@
         <v>0.19997409801805655</v>
       </c>
     </row>
-    <row r="252" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A252" t="s">
         <v>500</v>
       </c>
@@ -6568,7 +6568,7 @@
         <v>3.7478199229515192E-5</v>
       </c>
     </row>
-    <row r="253" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A253" t="s">
         <v>502</v>
       </c>
@@ -6586,7 +6586,7 @@
         <v>1.2031589684685495E-5</v>
       </c>
     </row>
-    <row r="254" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A254" t="s">
         <v>503</v>
       </c>
@@ -6604,7 +6604,7 @@
         <v>1.4381655238309811E-2</v>
       </c>
     </row>
-    <row r="255" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A255" t="s">
         <v>504</v>
       </c>
@@ -6622,7 +6622,7 @@
         <v>4.9074287069283875E-3</v>
       </c>
     </row>
-    <row r="256" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A256" t="s">
         <v>505</v>
       </c>
@@ -6640,7 +6640,7 @@
         <v>7.579439881164488E-3</v>
       </c>
     </row>
-    <row r="257" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A257" t="s">
         <v>506</v>
       </c>
@@ -6658,7 +6658,7 @@
         <v>1.2319201538785539E-2</v>
       </c>
     </row>
-    <row r="258" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A258" t="s">
         <v>507</v>
       </c>
@@ -6676,7 +6676,7 @@
         <v>5.5354856646011162E-2</v>
       </c>
     </row>
-    <row r="259" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A259" t="s">
         <v>508</v>
       </c>
@@ -6694,7 +6694,7 @@
         <v>3.060374014899734E-2</v>
       </c>
     </row>
-    <row r="260" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A260" t="s">
         <v>509</v>
       </c>
@@ -6712,7 +6712,7 @@
         <v>3.5400788925328053E-2</v>
       </c>
     </row>
-    <row r="261" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A261" t="s">
         <v>510</v>
       </c>
@@ -6730,7 +6730,7 @@
         <v>1.6604966693385109E-3</v>
       </c>
     </row>
-    <row r="262" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A262" t="s">
         <v>511</v>
       </c>
@@ -6748,7 +6748,7 @@
         <v>1.107174880230615E-3</v>
       </c>
     </row>
-    <row r="263" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A263" t="s">
         <v>512</v>
       </c>
@@ -6766,7 +6766,7 @@
         <v>7.8092637299048782E-3</v>
       </c>
     </row>
-    <row r="264" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A264" t="s">
         <v>513</v>
       </c>
@@ -6784,7 +6784,7 @@
         <v>2.9201116197698187E-2</v>
       </c>
     </row>
-    <row r="265" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A265" t="s">
         <v>514</v>
       </c>
@@ -6802,7 +6802,7 @@
         <v>1.4002759856788772E-2</v>
       </c>
     </row>
-    <row r="266" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A266" t="s">
         <v>515</v>
       </c>
@@ -6820,7 +6820,7 @@
         <v>1.0078376507246956E-2</v>
       </c>
     </row>
-    <row r="267" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A267" t="s">
         <v>516</v>
       </c>
@@ -6838,7 +6838,7 @@
         <v>0.12151148407082195</v>
       </c>
     </row>
-    <row r="268" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A268" t="s">
         <v>517</v>
       </c>
@@ -6856,7 +6856,7 @@
         <v>3.340044404852946E-2</v>
       </c>
     </row>
-    <row r="269" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A269" t="s">
         <v>518</v>
       </c>
@@ -6874,7 +6874,7 @@
         <v>7.1206225045451115E-3</v>
       </c>
     </row>
-    <row r="270" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A270" t="s">
         <v>519</v>
       </c>
@@ -6892,7 +6892,7 @@
         <v>3.7645682367898948E-3</v>
       </c>
     </row>
-    <row r="271" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A271" t="s">
         <v>520</v>
       </c>
@@ -6910,7 +6910,7 @@
         <v>2.9745351344251615E-3</v>
       </c>
     </row>
-    <row r="272" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A272" t="s">
         <v>521</v>
       </c>
@@ -6928,7 +6928,7 @@
         <v>2.474911379226509E-2</v>
       </c>
     </row>
-    <row r="273" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A273" t="s">
         <v>522</v>
       </c>
@@ -6946,7 +6946,7 @@
         <v>1.5755072911621121E-2</v>
       </c>
     </row>
-    <row r="274" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A274" t="s">
         <v>523</v>
       </c>
@@ -6964,7 +6964,7 @@
         <v>1.6383002588794681E-3</v>
       </c>
     </row>
-    <row r="275" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:5" x14ac:dyDescent="0.2">
       <c r="C275">
         <v>100</v>
       </c>
@@ -6972,7 +6972,7 @@
         <v>99.999999999999943</v>
       </c>
     </row>
-    <row r="276" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A276" s="3"/>
       <c r="B276" s="3"/>
     </row>

</xml_diff>